<commit_message>
migrate: add S28 P1 metadata to existing XLSX sheets
</commit_message>
<xml_diff>
--- a/crew_102.xlsx
+++ b/crew_102.xlsx
@@ -8,6 +8,7 @@
   </bookViews>
   <sheets>
     <sheet name="2026-07-16" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="2026-07-17" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -452,7 +453,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Crew: Blood Brothers (102)</t>
+          <t>Crew: Blood Brothers (102) | S28 P1</t>
         </is>
       </c>
     </row>
@@ -1403,6 +1404,992 @@
       </c>
       <c r="D43" s="5" t="n">
         <v>1475</v>
+      </c>
+      <c r="E43" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A2:E2"/>
+    <mergeCell ref="A1:E1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E43"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="25" customWidth="1" min="1" max="1"/>
+    <col width="9" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="9" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Crew: Blood Brothers (102) | S28 P1</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-07-17 13:54:08</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Dmg</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Daily Dmg</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>Boss Kills</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>Daily Kills</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Harimukun</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="n">
+        <v>748437</v>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>+85041</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="n">
+        <v>3563</v>
+      </c>
+      <c r="E4" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>NAOR</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="n">
+        <v>391577</v>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>+55362</t>
+        </is>
+      </c>
+      <c r="D5" s="5" t="n">
+        <v>1800</v>
+      </c>
+      <c r="E5" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>DangerousEX</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="n">
+        <v>554189</v>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>+73255</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="n">
+        <v>2642</v>
+      </c>
+      <c r="E6" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>X y l o t a [NvL]</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="n">
+        <v>488807</v>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>+146949</t>
+        </is>
+      </c>
+      <c r="D7" s="5" t="n">
+        <v>2205</v>
+      </c>
+      <c r="E7" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>Andrey</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="n">
+        <v>418271</v>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>+113169</t>
+        </is>
+      </c>
+      <c r="D8" s="5" t="n">
+        <v>1993</v>
+      </c>
+      <c r="E8" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>H U N T E R</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="n">
+        <v>531666</v>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>+86862</t>
+        </is>
+      </c>
+      <c r="D9" s="5" t="n">
+        <v>2526</v>
+      </c>
+      <c r="E9" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>SB ELISEUS</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="n">
+        <v>568086</v>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>+83310</t>
+        </is>
+      </c>
+      <c r="D10" s="5" t="n">
+        <v>2705</v>
+      </c>
+      <c r="E10" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>Toka Senju™</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="n">
+        <v>385937</v>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>+102157</t>
+        </is>
+      </c>
+      <c r="D11" s="5" t="n">
+        <v>1837</v>
+      </c>
+      <c r="E11" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>The prince JI OF NY</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="n">
+        <v>383480</v>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>+102777</t>
+        </is>
+      </c>
+      <c r="D12" s="5" t="n">
+        <v>1826</v>
+      </c>
+      <c r="E12" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>SNC | Conrad</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="n">
+        <v>271461</v>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>+92961</t>
+        </is>
+      </c>
+      <c r="D13" s="5" t="n">
+        <v>1294</v>
+      </c>
+      <c r="E13" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>YE Brandy</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="n">
+        <v>635089</v>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>+138400</t>
+        </is>
+      </c>
+      <c r="D14" s="5" t="n">
+        <v>3022</v>
+      </c>
+      <c r="E14" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>Kosaki</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="n">
+        <v>496666</v>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>+98625</t>
+        </is>
+      </c>
+      <c r="D15" s="5" t="n">
+        <v>2364</v>
+      </c>
+      <c r="E15" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>Snoopy | Kokyutosu</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="n">
+        <v>564307</v>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>+87777</t>
+        </is>
+      </c>
+      <c r="D16" s="5" t="n">
+        <v>2525</v>
+      </c>
+      <c r="E16" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>Pencilgon</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="n">
+        <v>533754</v>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>+131617</t>
+        </is>
+      </c>
+      <c r="D17" s="5" t="n">
+        <v>2542</v>
+      </c>
+      <c r="E17" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>The ProfessorX</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="n">
+        <v>412098</v>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>+96123</t>
+        </is>
+      </c>
+      <c r="D18" s="5" t="n">
+        <v>1960</v>
+      </c>
+      <c r="E18" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>Nabila|Fortuners</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="n">
+        <v>419960</v>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>+42781</t>
+        </is>
+      </c>
+      <c r="D19" s="5" t="n">
+        <v>2001</v>
+      </c>
+      <c r="E19" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>San Pate Té</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="n">
+        <v>552895</v>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>+61042</t>
+        </is>
+      </c>
+      <c r="D20" s="5" t="n">
+        <v>2469</v>
+      </c>
+      <c r="E20" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>Ryujin Senju™</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="n">
+        <v>568551</v>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>+71678</t>
+        </is>
+      </c>
+      <c r="D21" s="5" t="n">
+        <v>2663</v>
+      </c>
+      <c r="E21" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>Sabrina Carpenter</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="n">
+        <v>569878</v>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>+60550</t>
+        </is>
+      </c>
+      <c r="D22" s="5" t="n">
+        <v>2540</v>
+      </c>
+      <c r="E22" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>Kiroi Senko</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="n">
+        <v>301113</v>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>+86070</t>
+        </is>
+      </c>
+      <c r="D23" s="5" t="n">
+        <v>1434</v>
+      </c>
+      <c r="E23" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>NPC | SNOOPY</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="n">
+        <v>565295</v>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>+79156</t>
+        </is>
+      </c>
+      <c r="D24" s="5" t="n">
+        <v>2530</v>
+      </c>
+      <c r="E24" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nitro </t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="n">
+        <v>417227</v>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>+102771</t>
+        </is>
+      </c>
+      <c r="D25" s="5" t="n">
+        <v>1987</v>
+      </c>
+      <c r="E25" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>Flarekaze |Fortuners</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="n">
+        <v>606289</v>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>+44460</t>
+        </is>
+      </c>
+      <c r="D26" s="5" t="n">
+        <v>2885</v>
+      </c>
+      <c r="E26" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>Aldrin</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="n">
+        <v>447829</v>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>+130100</t>
+        </is>
+      </c>
+      <c r="D27" s="5" t="n">
+        <v>2133</v>
+      </c>
+      <c r="E27" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>YinRaku ™</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="n">
+        <v>332672</v>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>+54792</t>
+        </is>
+      </c>
+      <c r="D28" s="5" t="n">
+        <v>1514</v>
+      </c>
+      <c r="E28" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>~Pria_SoL0~</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="n">
+        <v>487885</v>
+      </c>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>+136434</t>
+        </is>
+      </c>
+      <c r="D29" s="5" t="n">
+        <v>2325</v>
+      </c>
+      <c r="E29" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>BlacKObito O</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="n">
+        <v>397397</v>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>+115698</t>
+        </is>
+      </c>
+      <c r="D30" s="5" t="n">
+        <v>1894</v>
+      </c>
+      <c r="E30" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>FEARLESS</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="n">
+        <v>388104</v>
+      </c>
+      <c r="C31" s="5" t="inlineStr">
+        <is>
+          <t>+57315</t>
+        </is>
+      </c>
+      <c r="D31" s="5" t="n">
+        <v>1673</v>
+      </c>
+      <c r="E31" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>zDexTerx</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="n">
+        <v>601479</v>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>+198145</t>
+        </is>
+      </c>
+      <c r="D32" s="5" t="n">
+        <v>2704</v>
+      </c>
+      <c r="E32" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>SharinganKniGhT</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="n">
+        <v>258100</v>
+      </c>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D33" s="5" t="n">
+        <v>1229</v>
+      </c>
+      <c r="E33" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>Armando</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="n">
+        <v>408877</v>
+      </c>
+      <c r="C34" s="5" t="inlineStr">
+        <is>
+          <t>+110683</t>
+        </is>
+      </c>
+      <c r="D34" s="5" t="n">
+        <v>1949</v>
+      </c>
+      <c r="E34" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>Ryujin 2ND</t>
+        </is>
+      </c>
+      <c r="B35" s="5" t="n">
+        <v>561879</v>
+      </c>
+      <c r="C35" s="5" t="inlineStr">
+        <is>
+          <t>+82807</t>
+        </is>
+      </c>
+      <c r="D35" s="5" t="n">
+        <v>2630</v>
+      </c>
+      <c r="E35" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="inlineStr">
+        <is>
+          <t>ANBU | HERO NICO 15</t>
+        </is>
+      </c>
+      <c r="B36" s="5" t="n">
+        <v>300753</v>
+      </c>
+      <c r="C36" s="5" t="inlineStr">
+        <is>
+          <t>+84906</t>
+        </is>
+      </c>
+      <c r="D36" s="5" t="n">
+        <v>1433</v>
+      </c>
+      <c r="E36" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="4" t="inlineStr">
+        <is>
+          <t>BlacKEucresia Ó</t>
+        </is>
+      </c>
+      <c r="B37" s="5" t="n">
+        <v>374576</v>
+      </c>
+      <c r="C37" s="5" t="inlineStr">
+        <is>
+          <t>+92882</t>
+        </is>
+      </c>
+      <c r="D37" s="5" t="n">
+        <v>1781</v>
+      </c>
+      <c r="E37" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="4" t="inlineStr">
+        <is>
+          <t>RS | Oboy Max</t>
+        </is>
+      </c>
+      <c r="B38" s="5" t="n">
+        <v>424198</v>
+      </c>
+      <c r="C38" s="5" t="inlineStr">
+        <is>
+          <t>+101990</t>
+        </is>
+      </c>
+      <c r="D38" s="5" t="n">
+        <v>2018</v>
+      </c>
+      <c r="E38" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t>Aiah</t>
+        </is>
+      </c>
+      <c r="B39" s="5" t="n">
+        <v>518039</v>
+      </c>
+      <c r="C39" s="5" t="inlineStr">
+        <is>
+          <t>+68301</t>
+        </is>
+      </c>
+      <c r="D39" s="5" t="n">
+        <v>2468</v>
+      </c>
+      <c r="E39" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t>Breaker MAX</t>
+        </is>
+      </c>
+      <c r="B40" s="5" t="n">
+        <v>358784</v>
+      </c>
+      <c r="C40" s="5" t="inlineStr">
+        <is>
+          <t>+114022</t>
+        </is>
+      </c>
+      <c r="D40" s="5" t="n">
+        <v>1709</v>
+      </c>
+      <c r="E40" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="4" t="inlineStr">
+        <is>
+          <t>[R23] Cub †</t>
+        </is>
+      </c>
+      <c r="B41" s="5" t="n">
+        <v>482531</v>
+      </c>
+      <c r="C41" s="5" t="inlineStr">
+        <is>
+          <t>+113520</t>
+        </is>
+      </c>
+      <c r="D41" s="5" t="n">
+        <v>2299</v>
+      </c>
+      <c r="E41" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="4" t="inlineStr">
+        <is>
+          <t>RS | Oboy Lite</t>
+        </is>
+      </c>
+      <c r="B42" s="5" t="n">
+        <v>375874</v>
+      </c>
+      <c r="C42" s="5" t="inlineStr">
+        <is>
+          <t>+97236</t>
+        </is>
+      </c>
+      <c r="D42" s="5" t="n">
+        <v>1791</v>
+      </c>
+      <c r="E42" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="4" t="inlineStr">
+        <is>
+          <t>Haise</t>
+        </is>
+      </c>
+      <c r="B43" s="5" t="n">
+        <v>374221</v>
+      </c>
+      <c r="C43" s="5" t="inlineStr">
+        <is>
+          <t>+50916</t>
+        </is>
+      </c>
+      <c r="D43" s="5" t="n">
+        <v>1719</v>
       </c>
       <c r="E43" s="5" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
fix: correct phase labels in excel A1 cells
</commit_message>
<xml_diff>
--- a/crew_102.xlsx
+++ b/crew_102.xlsx
@@ -1447,7 +1447,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Crew: Blood Brothers (102) | S28 P1</t>
+          <t>Crew: Blood Brothers (102) | S28 P2</t>
         </is>
       </c>
     </row>
@@ -4403,7 +4403,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Crew: Blood Brothers (102) | S28 P2</t>
+          <t>Crew: Blood Brothers (102) | S28 P1</t>
         </is>
       </c>
     </row>
@@ -5059,7 +5059,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Crew: Blood Brothers (102) | S28 P1</t>
+          <t>Crew: Blood Brothers (102) | S28 P2</t>
         </is>
       </c>
     </row>
@@ -6045,7 +6045,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Crew: Blood Brothers (102) | S28 P1</t>
+          <t>Crew: Blood Brothers (102) | S28 P2</t>
         </is>
       </c>
     </row>
@@ -7031,7 +7031,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Crew: Blood Brothers (102) | S28 P1</t>
+          <t>Crew: Blood Brothers (102) | S28 P2</t>
         </is>
       </c>
     </row>
@@ -8017,7 +8017,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Crew: Blood Brothers (102) | S28 P1</t>
+          <t>Crew: Blood Brothers (102) | S28 P2</t>
         </is>
       </c>
     </row>
@@ -9003,7 +9003,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Crew: Blood Brothers (102) | S28 P1</t>
+          <t>Crew: Blood Brothers (102) | S28 P2</t>
         </is>
       </c>
     </row>

</xml_diff>